<commit_message>
Add normal car specs dataset, Vercel Docker setup, collapsible specs panel, and custom reminder inputs
</commit_message>
<xml_diff>
--- a/backend/data/garages.xlsx
+++ b/backend/data/garages.xlsx
@@ -512,7 +512,7 @@
         <v>78.9941389</v>
       </c>
       <c r="G5" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         <v>79.1279209644177</v>
       </c>
       <c r="G8" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>79.0970650865062</v>
       </c>
       <c r="G11" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="12">
@@ -673,7 +673,7 @@
         <v>79.1383234124537</v>
       </c>
       <c r="G12" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="13">
@@ -696,7 +696,7 @@
         <v>79.1264600247829</v>
       </c>
       <c r="G13" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="14">
@@ -719,7 +719,7 @@
         <v>79.0417280423291</v>
       </c>
       <c r="G14" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="15">
@@ -765,7 +765,7 @@
         <v>79.1419424576708</v>
       </c>
       <c r="G16" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="17">

</xml_diff>